<commit_message>
fix: datas e porcentagem no formato brasileiro nos .xlsx
</commit_message>
<xml_diff>
--- a/dados/brutos/comercial_parceiros.xlsx
+++ b/dados/brutos/comercial_parceiros.xlsx
@@ -17,9 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -52,7 +53,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>

</xml_diff>